<commit_message>
(hel-1133) ajouter les indicateurs capacite dans le lisez moi de lexport excel
</commit_message>
<xml_diff>
--- a/public/templates/template_comparaison_SAN.xlsx
+++ b/public/templates/template_comparaison_SAN.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://catamaniacrm-my.sharepoint.com/personal/y_elhouakmi_catamania_com/Documents/Documents/DNum/Helios/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\schlaifa\projets\helios\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{78467E00-9E0B-4CF2-B9EB-D89DF4DDBF67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89141786-DFE5-429E-B2AC-0E33B484EAC3}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A46C86F-6A21-4401-A6C7-CACC3D178FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12240" yWindow="15984" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lisez-moi" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
   <si>
     <t>Indicateurs</t>
   </si>
@@ -1126,12 +1126,174 @@
 Hélios collecte ces données depuis le SI mutualisé des ARS DIAMANT « Décisionnel Inter-ARS pour la Maîtrise et l’Anticipation », outil décisionnel de pilotage centré sur la régulation de l’offre de soins, abordée sous les aspects des moyens humains, financiers, et productivité.</t>
     </r>
   </si>
+  <si>
+    <t>Nombre de lits Médecine</t>
+  </si>
+  <si>
+    <t>Nombre de lits PSY (Hospitalisation complète)</t>
+  </si>
+  <si>
+    <t>Nombre de lits SSR</t>
+  </si>
+  <si>
+    <t>Nombre de lits USLD</t>
+  </si>
+  <si>
+    <t>Nombre de lits Obstétrique</t>
+  </si>
+  <si>
+    <t>Nombre de lits Chirurgie</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Source : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SAE</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Permet de caractériser les capacités d’accueil de l’établissement et les alternatives à l’hospitalisation conventionnelle avec nuitée dont il dispose.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Fréquence :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Annuelle</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Mode de calcul :
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Nombre de lits MCO : Le nombre de lits installés correspond aux lits intégrés au sein de services d’hospitalisation complète, y compris l’hospitalisation de semaine.
+Nombre de places MCO : Le nombre de places installées au 31 décembre de l’année est égal au nombre de patients pouvant être accueillis en même temps.
+Nombre de lits SSR : Le nombre de lits installés au 31 décembre de l’année est égal à la somme du nombre de lits en état d’accueillir des malades.
+Nombre de places SSR : Le nombre de places installées au 31 décembre de l’année en hospitalisation à temps partiel de jour ou de nuit est égal au nombre de patients pouvant être accueillis en même temps.
+Nombre de lits PSY (capacité en HC) : le nombre de lits installés au 31 décembre de l’année est égal à la somme du nombre de lits en état d’accueillir des malades et du nombre de de patients pouvant être pris en charge simultanément en hospitalisation à domicile (HAD).
+Nombre de places PSY : Le nombre de places installées au 31 décembre de l’année en hospitalisation à temps partiel de jour ou de nuit est égal au nombre de patients pouvant être accueillis en même temps, hors prise en charge ambulatoire.
+Nombre de lits USLD : Le nombre de lits installés au 31 décembre de l’année est égal à la somme du nombre de lits en état d’accueillir des malades.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Source(s) :
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Statistique annuelle des établissements de santé (SAE) - Direction de la Recherche, des Études, de l’Évaluation et des Statistiques (DREES).
+La Statistique annuelle des établissements de santé (SAE) est une enquête administrative exhaustive obligatoire, réalisée chaque année par la DREES auprès de tous les établissements de santé de France, pour recueillir des informations sur leur activité, leurs capacités, leurs équipements, et leurs personnel médicaux et non-médicaux.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hélios collecte ces données depuis le SI mutualisé des ARS DIAMANT « Décisionnel Inter-ARS pour la Maîtrise et l’Anticipation. », outil décisionnel de pilotage centré sur la régulation de l’offre de soins, abordée sous les aspects des moyens humains, financiers, et productivité.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1160,6 +1322,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1181,7 +1350,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1203,6 +1372,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1543,15 +1715,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{587C9ED0-279B-44AC-9485-AC6832055B1B}">
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C23"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.19921875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="20.09765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="187.59765625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="21.25" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="187.625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1562,176 +1734,224 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="108" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="31.2" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>6</v>
+        <v>42</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="6"/>
     </row>
-    <row r="4" spans="1:3" ht="309" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="95.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="6"/>
     </row>
-    <row r="5" spans="1:3" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="136.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+      <c r="B5" s="7"/>
+      <c r="C5" s="6"/>
+    </row>
+    <row r="6" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="6"/>
     </row>
-    <row r="7" spans="1:3" ht="274.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="6"/>
+    </row>
+    <row r="8" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="7"/>
+      <c r="C9" s="8"/>
+    </row>
+    <row r="10" spans="1:3" ht="309" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="8"/>
+    </row>
+    <row r="11" spans="1:3" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="136.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="7"/>
+      <c r="C12" s="6"/>
+    </row>
+    <row r="13" spans="1:3" ht="274.89999999999998" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="327.60000000000002" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+    <row r="14" spans="1:3" ht="315" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B14" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C14" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="156" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+    <row r="15" spans="1:3" ht="157.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="156" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="156" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="171.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="171.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="240" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="249.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
-        <v>31</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="218.4" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="157.5" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="249.6" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="157.5" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="173.25" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="173.25" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="240" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="252" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="220.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="252" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>36</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B5:B6"/>
+  <mergeCells count="6">
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="B2:B7"/>
+    <mergeCell ref="C2:C7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1741,7 +1961,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Hel 1133/ajout capacite san pour comparaison (#1192)
* (hel-1133) ajout des indicateurs capacite sanitaire dans la comparaison

* (hel-1133) ajouter les indicateurs capacite dans le lisez moi de lexport excel

* (hel-1133) export des indicateurs capacite sanitaire
</commit_message>
<xml_diff>
--- a/public/templates/template_comparaison_SAN.xlsx
+++ b/public/templates/template_comparaison_SAN.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://catamaniacrm-my.sharepoint.com/personal/y_elhouakmi_catamania_com/Documents/Documents/DNum/Helios/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\schlaifa\projets\helios\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{78467E00-9E0B-4CF2-B9EB-D89DF4DDBF67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89141786-DFE5-429E-B2AC-0E33B484EAC3}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A46C86F-6A21-4401-A6C7-CACC3D178FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12240" yWindow="15984" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lisez-moi" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
   <si>
     <t>Indicateurs</t>
   </si>
@@ -1126,12 +1126,174 @@
 Hélios collecte ces données depuis le SI mutualisé des ARS DIAMANT « Décisionnel Inter-ARS pour la Maîtrise et l’Anticipation », outil décisionnel de pilotage centré sur la régulation de l’offre de soins, abordée sous les aspects des moyens humains, financiers, et productivité.</t>
     </r>
   </si>
+  <si>
+    <t>Nombre de lits Médecine</t>
+  </si>
+  <si>
+    <t>Nombre de lits PSY (Hospitalisation complète)</t>
+  </si>
+  <si>
+    <t>Nombre de lits SSR</t>
+  </si>
+  <si>
+    <t>Nombre de lits USLD</t>
+  </si>
+  <si>
+    <t>Nombre de lits Obstétrique</t>
+  </si>
+  <si>
+    <t>Nombre de lits Chirurgie</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Source : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SAE</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Permet de caractériser les capacités d’accueil de l’établissement et les alternatives à l’hospitalisation conventionnelle avec nuitée dont il dispose.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Fréquence :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Annuelle</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Mode de calcul :
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Nombre de lits MCO : Le nombre de lits installés correspond aux lits intégrés au sein de services d’hospitalisation complète, y compris l’hospitalisation de semaine.
+Nombre de places MCO : Le nombre de places installées au 31 décembre de l’année est égal au nombre de patients pouvant être accueillis en même temps.
+Nombre de lits SSR : Le nombre de lits installés au 31 décembre de l’année est égal à la somme du nombre de lits en état d’accueillir des malades.
+Nombre de places SSR : Le nombre de places installées au 31 décembre de l’année en hospitalisation à temps partiel de jour ou de nuit est égal au nombre de patients pouvant être accueillis en même temps.
+Nombre de lits PSY (capacité en HC) : le nombre de lits installés au 31 décembre de l’année est égal à la somme du nombre de lits en état d’accueillir des malades et du nombre de de patients pouvant être pris en charge simultanément en hospitalisation à domicile (HAD).
+Nombre de places PSY : Le nombre de places installées au 31 décembre de l’année en hospitalisation à temps partiel de jour ou de nuit est égal au nombre de patients pouvant être accueillis en même temps, hors prise en charge ambulatoire.
+Nombre de lits USLD : Le nombre de lits installés au 31 décembre de l’année est égal à la somme du nombre de lits en état d’accueillir des malades.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Source(s) :
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Statistique annuelle des établissements de santé (SAE) - Direction de la Recherche, des Études, de l’Évaluation et des Statistiques (DREES).
+La Statistique annuelle des établissements de santé (SAE) est une enquête administrative exhaustive obligatoire, réalisée chaque année par la DREES auprès de tous les établissements de santé de France, pour recueillir des informations sur leur activité, leurs capacités, leurs équipements, et leurs personnel médicaux et non-médicaux.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hélios collecte ces données depuis le SI mutualisé des ARS DIAMANT « Décisionnel Inter-ARS pour la Maîtrise et l’Anticipation. », outil décisionnel de pilotage centré sur la régulation de l’offre de soins, abordée sous les aspects des moyens humains, financiers, et productivité.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1160,6 +1322,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1181,7 +1350,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1203,6 +1372,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1543,15 +1715,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{587C9ED0-279B-44AC-9485-AC6832055B1B}">
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C23"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.19921875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="20.09765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="187.59765625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="21.25" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="187.625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1562,176 +1734,224 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="108" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="31.2" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>6</v>
+        <v>42</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="6"/>
     </row>
-    <row r="4" spans="1:3" ht="309" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="95.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="6"/>
     </row>
-    <row r="5" spans="1:3" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="136.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+      <c r="B5" s="7"/>
+      <c r="C5" s="6"/>
+    </row>
+    <row r="6" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="6"/>
     </row>
-    <row r="7" spans="1:3" ht="274.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="6"/>
+    </row>
+    <row r="8" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="7"/>
+      <c r="C9" s="8"/>
+    </row>
+    <row r="10" spans="1:3" ht="309" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="8"/>
+    </row>
+    <row r="11" spans="1:3" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="136.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="7"/>
+      <c r="C12" s="6"/>
+    </row>
+    <row r="13" spans="1:3" ht="274.89999999999998" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="327.60000000000002" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+    <row r="14" spans="1:3" ht="315" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B14" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C14" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="156" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+    <row r="15" spans="1:3" ht="157.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="156" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="156" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="171.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="171.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="240" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="249.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
-        <v>31</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="218.4" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="157.5" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="249.6" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="157.5" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="173.25" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="173.25" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="240" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="252" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="220.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="252" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>36</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B5:B6"/>
+  <mergeCells count="6">
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="B2:B7"/>
+    <mergeCell ref="C2:C7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1741,7 +1961,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>